<commit_message>
Ai tool started working
</commit_message>
<xml_diff>
--- a/export/bugs_report.xlsx
+++ b/export/bugs_report.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,17 +27,28 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0018181b"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,13 +56,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E4E4E7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E4E4E7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E4E4E7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E4E4E7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,10 +450,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>S.No</t>
@@ -465,6 +509,142 @@
         <is>
           <t>Screenshot</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Page Not Reachable / Connection Failed</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>1. Open browser
+2. Navigate to https://broken-link-checker.com</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Page should load successfully without errors</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Connection failed: HTTPSConnectionPool(host='broken-link-checker.com', port=443): Max retries exceeded with url: / (Cau</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Page Not Found (404)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>1. Open browser
+2. Navigate to https://httpbin.org/status/404</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Page should exist and load correctly</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Server returned HTTP 404 - Page not found</t>
+        </is>
+      </c>
+      <c r="I3" s="3">
+        <f>HYPERLINK("screenshots/scan_httpbin.org_status_404_20260401_200613.png","Open Screenshot")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Internal Server Error (500)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1. Open browser
+2. Navigate to https://httpbin.org/status/500</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Page should display content correctly</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Server returned HTTP 500 Internal Server Error</t>
+        </is>
+      </c>
+      <c r="I4" s="3">
+        <f>HYPERLINK("screenshots/scan_httpbin.org_status_500_20260401_201542.png","Open Screenshot")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>